<commit_message>
Enterprise hardening pass: Mega Project 1 (Underwriting & Approval Intelligence) built and verified; suite corrected to its final 5-Mega-Project scope. See CHANGELOG.md for full disclosure of every fix.
</commit_message>
<xml_diff>
--- a/01_mega_project_1_underwriting_approval/sample_reports/SAMPLE_mp1_executive_report.xlsx
+++ b/01_mega_project_1_underwriting_approval/sample_reports/SAMPLE_mp1_executive_report.xlsx
@@ -578,7 +578,7 @@
     <row r="5">
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>$364,691</t>
+          <t>$364,625</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
     <row r="8">
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>$1,823,454</t>
+          <t>$1,823,126</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>333165.77</v>
+        <v>334125.17</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>19525</v>
+        <v>18500</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -826,7 +826,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NOT RECOMMENDED FOR PRODUCTION YET — failed: auc_ci_lower_above_random (this is a separate, stricter statistical-robustness gate, distinct from the structural pipeline integrity checks reported elsewhere in this notebook's output; failing here does not indicate a code defect, and passing all integrity checks does not imply this gate passed -- expected and informational on small or noisy real/synthetic samples, see this problem's MODEL_CARD.md)</t>
+          <t>RECOMMENDED FOR PRODUCTION</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -840,13 +840,13 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>333165.76875</v>
+        <v>334125.16875</v>
       </c>
       <c r="J2" t="n">
         <v>259486224</v>
       </c>
       <c r="K2" t="n">
-        <v>14.3</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -862,7 +862,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -881,13 +881,13 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>19525</v>
+        <v>18500</v>
       </c>
       <c r="J3" t="n">
         <v>142039488</v>
       </c>
       <c r="K3" t="n">
-        <v>29.9</v>
+        <v>27.6</v>
       </c>
     </row>
     <row r="4">
@@ -908,7 +908,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NOT RECOMMENDED FOR PRODUCTION YET — failed: mean_calibration_gap_acceptable (this is a separate, stricter statistical-robustness gate, distinct from the structural pipeline integrity checks reported elsewhere in this notebook's output; failing here does not indicate a code defect, and passing all integrity checks does not imply this gate passed -- expected and informational on small or noisy real/synthetic samples, see this problem's MODEL_CARD.md)</t>
+          <t>RECOMMENDED FOR PRODUCTION</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -928,7 +928,7 @@
         <v>1726180608</v>
       </c>
       <c r="K4" t="n">
-        <v>6.7</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="5">
@@ -969,7 +969,7 @@
         <v>1726180495.26</v>
       </c>
       <c r="K5" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="6">
@@ -1010,7 +1010,7 @@
         <v>944202702.8599979</v>
       </c>
       <c r="K6" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1074,7 +1074,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>30390.89739583333</v>
+        <v>30385.43072916667</v>
       </c>
     </row>
     <row r="3">
@@ -1087,7 +1087,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>182345.384375</v>
+        <v>182312.584375</v>
       </c>
     </row>
     <row r="4">
@@ -1100,7 +1100,7 @@
         <v>12</v>
       </c>
       <c r="C4" t="n">
-        <v>364690.76875</v>
+        <v>364625.16875</v>
       </c>
     </row>
     <row r="5">
@@ -1113,7 +1113,7 @@
         <v>24</v>
       </c>
       <c r="C5" t="n">
-        <v>729381.5375</v>
+        <v>729250.3375</v>
       </c>
     </row>
     <row r="6">
@@ -1126,7 +1126,7 @@
         <v>36</v>
       </c>
       <c r="C6" t="n">
-        <v>1094072.30625</v>
+        <v>1093875.50625</v>
       </c>
     </row>
     <row r="7">
@@ -1139,7 +1139,7 @@
         <v>60</v>
       </c>
       <c r="C7" t="n">
-        <v>1823453.84375</v>
+        <v>1823125.84375</v>
       </c>
     </row>
   </sheetData>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Problem 1 — Credit Default Prediction: NOT RECOMMENDED FOR PRODUCTION YET</t>
+          <t>Problem 1 — Credit Default Prediction: RECOMMENDED FOR PRODUCTION</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>$333,165.77 real illustrative benefit</t>
+          <t>$334,125.17 real illustrative benefit</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -1358,12 +1358,12 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Problem 3 — Loan Application Approval uses RandomForest and passed 18/18 PASS real integrity self-checks on its most recent run.</t>
+          <t>Problem 3 — Loan Application Approval uses CatBoost and passed 18/18 PASS real integrity self-checks on its most recent run.</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>$19,525.00 real illustrative benefit</t>
+          <t>$18,500.00 real illustrative benefit</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Problem 4 — Credit Score Estimation: NOT RECOMMENDED FOR PRODUCTION YET</t>
+          <t>Problem 4 — Credit Score Estimation: RECOMMENDED FOR PRODUCTION</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">

</xml_diff>